<commit_message>
Copilot CLI session c2380152-334c-4c4a-990f-333f1ceda4a2 changes
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,13 +494,59 @@
           <t>pradhan04_</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>gggggggggggg</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>444444444444444</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>hhhhhhhhhhhhhhhhhhhhh@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>llllllllllllll</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>gggggggggggg_c002</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$hNOfWFAPdqSs5Ees$44e4241ed49f35a4a9a0ccbca22302476fdf1e3314358bfca4096673c4b71e28769de65c52ba012eb30e7d9d15fcbb75f6574986746d3bac9a3a21965856a520</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>

</xml_diff>

<commit_message>
chore: remove gitignore and add data files and python cache artifacts
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,13 +494,59 @@
           <t>pradhan04_</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>gggggggggggg</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>444444444444444</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>hhhhhhhhhhhhhhhhhhhhh@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>llllllllllllll</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>gggggggggggg_c002</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$hNOfWFAPdqSs5Ees$44e4241ed49f35a4a9a0ccbca22302476fdf1e3314358bfca4096673c4b71e28769de65c52ba012eb30e7d9d15fcbb75f6574986746d3bac9a3a21965856a520</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>

</xml_diff>

<commit_message>
Add static portfolio landing page and Flask integration
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,95 +460,6 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>reg_date</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>C001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Umashankar Pradhan</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>+919668797558</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>umashankarpradhan138@gmail.com</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Dighalo, nimapada, puri</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>pradhan04_</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>C002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>gggggggggggg</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>444444444444444</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>hhhhhhhhhhhhhhhhhhhhh@gmail.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>llllllllllllll</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>gggggggggggg_c002</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>scrypt:32768:8:1$hNOfWFAPdqSs5Ees$44e4241ed49f35a4a9a0ccbca22302476fdf1e3314358bfca4096673c4b71e28769de65c52ba012eb30e7d9d15fcbb75f6574986746d3bac9a3a21965856a520</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update clients spreadsheet with test client
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,7 +484,6 @@
           <t>test@example.com</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>testclient_c001</t>
@@ -503,6 +502,45 @@
       <c r="I2" t="inlineStr">
         <is>
           <t>2026-07-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Browser Test Client</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>browsertest</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$xXqKyLChYwvpeBOg$89547adf5c430f3eaf1638bd927aad0a94f488876f0b90420ac912f15a3176a93439240d1b158cebbf5900f46382c2719f8df990a3f052e80ac53ac39733dac3</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
         </is>
       </c>
     </row>

</xml_diff>